<commit_message>
Fix Excel chart titles overlapping plot and add axis titles
- Set chart title overlay=0 so the title sits above the plot instead of on
  top of the bars/lines
- Add category/value axis titles (Year/Month/Ward vs. Units issued) and force
  axes visible (delete=0) on the bar and line charts
- Slightly taller charts for clearer layout
- Rebuild template + single-file BloodBankStatistics.html

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0112qHiB1UY5umc5XsmN5SzT
</commit_message>
<xml_diff>
--- a/tools/template.xlsx
+++ b/tools/template.xlsx
@@ -274,6 +274,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <pieChart>
@@ -345,7 +346,7 @@
       </pieChart>
     </plotArea>
     <legend>
-      <legendPos val="r"/>
+      <legendPos val="b"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -370,6 +371,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>
@@ -492,7 +494,24 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Year</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+          <overlay val="0"/>
+        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
@@ -503,14 +522,32 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Units issued</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+          <overlay val="0"/>
+        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
       </valAx>
     </plotArea>
     <legend>
-      <legendPos val="r"/>
+      <legendPos val="b"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -535,6 +572,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>
@@ -658,7 +696,24 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Ward / Floor</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+          <overlay val="0"/>
+        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
@@ -669,15 +724,32 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Units issued</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+          <overlay val="0"/>
+        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
       </valAx>
     </plotArea>
     <legend>
-      <legendPos val="r"/>
+      <legendPos val="b"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -702,6 +774,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <lineChart>
@@ -859,7 +932,24 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Month</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+          <overlay val="0"/>
+        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
@@ -870,15 +960,32 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Units issued</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+          <overlay val="0"/>
+        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
       </valAx>
     </plotArea>
     <legend>
-      <legendPos val="r"/>
+      <legendPos val="b"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -922,7 +1029,7 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6480000" cy="2880000"/>
+    <ext cx="6480000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -949,7 +1056,7 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6480000" cy="3600000"/>
+    <ext cx="6480000" cy="3960000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -976,7 +1083,7 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7200000" cy="2880000"/>
+    <ext cx="7200000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>

</xml_diff>

<commit_message>
Add Transfusion Lab tests graphs to the exported files
- Styled analysis workbook: new "Lab Tests" sheet with three native Excel
  charts — lab tests per year (bar), counts by test (horizontal bar), and lab
  tests per month (line) — built into the embedded template and injected with
  live values at export; chart data ranges patched to the actual year/month
  counts
- Printable/PDF report: lab section now includes per-year and per-month charts
  alongside the by-test breakdown and table
- template-embed.js/meta and single-file build rebuilt

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0112qHiB1UY5umc5XsmN5SzT
</commit_message>
<xml_diff>
--- a/tools/template.xlsx
+++ b/tools/template.xlsx
@@ -11,6 +11,7 @@
     <sheet name="By Year" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="By Ward" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="By Month" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Lab Tests" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -993,6 +994,333 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Lab tests per year</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+      <overlay val="0"/>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="2A78D6"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Lab Tests'!$A$4:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Lab Tests'!$B$4:$B$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Year</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+          <overlay val="0"/>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Tests</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+          <overlay val="0"/>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Counts by test</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+      <overlay val="0"/>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="bar"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="1BAF7A"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Lab Tests'!$A$20:$A$42</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Lab Tests'!$B$20:$B$42</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Count</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+          <overlay val="0"/>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Lab tests per month</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+      <overlay val="0"/>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln w="20000">
+              <a:solidFill>
+                <a:srgbClr val="1BAF7A"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Lab Tests'!$A$47:$A$76</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Lab Tests'!$B$47:$B$76</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="0"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Month</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+          <overlay val="0"/>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Tests</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+          <overlay val="0"/>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -1093,6 +1421,77 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4680000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>18</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4680000" cy="3960000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>44</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7200000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -4060,4 +4459,1047 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C166"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Transfusion Lab tests</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Lab tests</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n"/>
+      <c r="B7" s="7" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="n"/>
+      <c r="B8" s="5" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n"/>
+      <c r="B9" s="7" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n"/>
+      <c r="B10" s="5" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n"/>
+      <c r="B11" s="7" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n"/>
+      <c r="B12" s="5" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n"/>
+      <c r="B13" s="7" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n"/>
+      <c r="B14" s="5" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n"/>
+      <c r="B15" s="7" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B16" s="17">
+        <f>SUM(B4:B15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Name of test</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>NO,SPECIMENS REC'D (IP)</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>NO,SPECIMENS REC'D (OP)</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>ABO&amp; RhD (IP)</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>ABO&amp; RhD (OP)</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Rh Weak D (OP)</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>Rh Weak D (IP)</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>DIRECT COOMBS (OP)</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>DIRECT COOMBS (IP)</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Ab SCREENING RT/37 (IP)</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Ab SCREENING RT/37 (OP)</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>PANEL (OP)</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>PANEL (IP)</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>TITRATION (IP)</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>TITRATION (OP)</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Ag TYPING RT (OP)</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>Ag TYPING RT (IP)</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Ag TYPING w/ AHG (IP)</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>Ag TYPING w/ AHG (OP)</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>X-MATCHING (IS)</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>X-MATCHING (AHG)</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Trnsfusion reaction</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>ELUTION</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Adsorption</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="18" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B43" s="17">
+        <f>SUM(B20:B42)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Lab tests</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Jan 2024</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>Feb 2024</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Mar 2024</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>Apr 2024</t>
+        </is>
+      </c>
+      <c r="B50" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>May 2024</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>Jun 2024</t>
+        </is>
+      </c>
+      <c r="B52" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Jul 2024</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>Aug 2024</t>
+        </is>
+      </c>
+      <c r="B54" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Sep 2024</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>Oct 2024</t>
+        </is>
+      </c>
+      <c r="B56" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Nov 2024</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>Dec 2024</t>
+        </is>
+      </c>
+      <c r="B58" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>Jan 2025</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>Feb 2025</t>
+        </is>
+      </c>
+      <c r="B60" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>Mar 2025</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>Apr 2025</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>May 2025</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="inlineStr">
+        <is>
+          <t>Jun 2025</t>
+        </is>
+      </c>
+      <c r="B64" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>Jul 2025</t>
+        </is>
+      </c>
+      <c r="B65" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="inlineStr">
+        <is>
+          <t>Sep 2025</t>
+        </is>
+      </c>
+      <c r="B66" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t>Oct 2025</t>
+        </is>
+      </c>
+      <c r="B67" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="inlineStr">
+        <is>
+          <t>Nov 2025</t>
+        </is>
+      </c>
+      <c r="B68" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>Dec 2025</t>
+        </is>
+      </c>
+      <c r="B69" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="inlineStr">
+        <is>
+          <t>Jan 2026</t>
+        </is>
+      </c>
+      <c r="B70" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t>Feb 2026</t>
+        </is>
+      </c>
+      <c r="B71" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="inlineStr">
+        <is>
+          <t>Mar 2026</t>
+        </is>
+      </c>
+      <c r="B72" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="B74" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="B75" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="B76" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="n"/>
+      <c r="B77" s="5" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="6" t="n"/>
+      <c r="B78" s="7" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="n"/>
+      <c r="B79" s="5" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="6" t="n"/>
+      <c r="B80" s="7" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="n"/>
+      <c r="B81" s="5" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="6" t="n"/>
+      <c r="B82" s="7" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="n"/>
+      <c r="B83" s="5" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="6" t="n"/>
+      <c r="B84" s="7" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="n"/>
+      <c r="B85" s="5" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="6" t="n"/>
+      <c r="B86" s="7" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="n"/>
+      <c r="B87" s="5" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="6" t="n"/>
+      <c r="B88" s="7" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="4" t="n"/>
+      <c r="B89" s="5" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="6" t="n"/>
+      <c r="B90" s="7" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="4" t="n"/>
+      <c r="B91" s="5" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="6" t="n"/>
+      <c r="B92" s="7" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="4" t="n"/>
+      <c r="B93" s="5" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="6" t="n"/>
+      <c r="B94" s="7" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="4" t="n"/>
+      <c r="B95" s="5" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="6" t="n"/>
+      <c r="B96" s="7" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="4" t="n"/>
+      <c r="B97" s="5" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="6" t="n"/>
+      <c r="B98" s="7" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="4" t="n"/>
+      <c r="B99" s="5" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="6" t="n"/>
+      <c r="B100" s="7" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="4" t="n"/>
+      <c r="B101" s="5" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="6" t="n"/>
+      <c r="B102" s="7" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="4" t="n"/>
+      <c r="B103" s="5" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="6" t="n"/>
+      <c r="B104" s="7" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="4" t="n"/>
+      <c r="B105" s="5" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="6" t="n"/>
+      <c r="B106" s="7" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="4" t="n"/>
+      <c r="B107" s="5" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="6" t="n"/>
+      <c r="B108" s="7" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="4" t="n"/>
+      <c r="B109" s="5" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="6" t="n"/>
+      <c r="B110" s="7" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="4" t="n"/>
+      <c r="B111" s="5" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="6" t="n"/>
+      <c r="B112" s="7" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="4" t="n"/>
+      <c r="B113" s="5" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="6" t="n"/>
+      <c r="B114" s="7" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="4" t="n"/>
+      <c r="B115" s="5" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="6" t="n"/>
+      <c r="B116" s="7" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="4" t="n"/>
+      <c r="B117" s="5" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="6" t="n"/>
+      <c r="B118" s="7" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="4" t="n"/>
+      <c r="B119" s="5" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="6" t="n"/>
+      <c r="B120" s="7" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="4" t="n"/>
+      <c r="B121" s="5" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="6" t="n"/>
+      <c r="B122" s="7" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="4" t="n"/>
+      <c r="B123" s="5" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="6" t="n"/>
+      <c r="B124" s="7" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="4" t="n"/>
+      <c r="B125" s="5" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="6" t="n"/>
+      <c r="B126" s="7" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="4" t="n"/>
+      <c r="B127" s="5" t="n"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="6" t="n"/>
+      <c r="B128" s="7" t="n"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="4" t="n"/>
+      <c r="B129" s="5" t="n"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="6" t="n"/>
+      <c r="B130" s="7" t="n"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="4" t="n"/>
+      <c r="B131" s="5" t="n"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="6" t="n"/>
+      <c r="B132" s="7" t="n"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="4" t="n"/>
+      <c r="B133" s="5" t="n"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="6" t="n"/>
+      <c r="B134" s="7" t="n"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="4" t="n"/>
+      <c r="B135" s="5" t="n"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="6" t="n"/>
+      <c r="B136" s="7" t="n"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="4" t="n"/>
+      <c r="B137" s="5" t="n"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="6" t="n"/>
+      <c r="B138" s="7" t="n"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="4" t="n"/>
+      <c r="B139" s="5" t="n"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="6" t="n"/>
+      <c r="B140" s="7" t="n"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="4" t="n"/>
+      <c r="B141" s="5" t="n"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="6" t="n"/>
+      <c r="B142" s="7" t="n"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="4" t="n"/>
+      <c r="B143" s="5" t="n"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="6" t="n"/>
+      <c r="B144" s="7" t="n"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="4" t="n"/>
+      <c r="B145" s="5" t="n"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="6" t="n"/>
+      <c r="B146" s="7" t="n"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="4" t="n"/>
+      <c r="B147" s="5" t="n"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="6" t="n"/>
+      <c r="B148" s="7" t="n"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="4" t="n"/>
+      <c r="B149" s="5" t="n"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="6" t="n"/>
+      <c r="B150" s="7" t="n"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="4" t="n"/>
+      <c r="B151" s="5" t="n"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="6" t="n"/>
+      <c r="B152" s="7" t="n"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="4" t="n"/>
+      <c r="B153" s="5" t="n"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="6" t="n"/>
+      <c r="B154" s="7" t="n"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="4" t="n"/>
+      <c r="B155" s="5" t="n"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="6" t="n"/>
+      <c r="B156" s="7" t="n"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="4" t="n"/>
+      <c r="B157" s="5" t="n"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="6" t="n"/>
+      <c r="B158" s="7" t="n"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="4" t="n"/>
+      <c r="B159" s="5" t="n"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="6" t="n"/>
+      <c r="B160" s="7" t="n"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="4" t="n"/>
+      <c r="B161" s="5" t="n"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="6" t="n"/>
+      <c r="B162" s="7" t="n"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="4" t="n"/>
+      <c r="B163" s="5" t="n"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="6" t="n"/>
+      <c r="B164" s="7" t="n"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="4" t="n"/>
+      <c r="B165" s="5" t="n"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="6" t="n"/>
+      <c r="B166" s="7" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>